<commit_message>
Add IT Home RSS source
</commit_message>
<xml_diff>
--- a/sources.xlsx
+++ b/sources.xlsx
@@ -400,7 +400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="32.5546875" customWidth="1" min="1" max="1"/>
@@ -2303,6 +2303,48 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>IT之家</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr">
+        <is>
+          <t>综合媒体</t>
+        </is>
+      </c>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>综合媒体</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>科技新闻</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>实时</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>IT之家科技资讯 RSS，覆盖科技、数码、互联网、软硬件与行业动态。</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>RSS: https://www.ithome.com/rss/</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>https://www.ithome.com/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>